<commit_message>
Quartz sync: Sep 9, 2025, 10:14 AM
</commit_message>
<xml_diff>
--- a/content/Notes/Biology/Labs/Excel/Lab 1.xlsx
+++ b/content/Notes/Biology/Labs/Excel/Lab 1.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gassandrid/VAULT/Notes/Biology/Labs/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E92522-17B3-7044-83E1-BD639D419FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C820872-849D-C04D-A0F1-673F3CDB534B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="740" windowWidth="34440" windowHeight="21540" activeTab="2" xr2:uid="{16F632E2-7B1C-374A-AA6C-9F513062A785}"/>
+    <workbookView xWindow="60" yWindow="740" windowWidth="34440" windowHeight="21540" activeTab="3" xr2:uid="{16F632E2-7B1C-374A-AA6C-9F513062A785}"/>
   </bookViews>
   <sheets>
     <sheet name="Chart1" sheetId="3" r:id="rId1"/>
     <sheet name="Chart2" sheetId="4" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="5" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Chart3" sheetId="6" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -967,37 +968,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
+    <c:autoTitleDeleted val="1"/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
@@ -1028,6 +999,99 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:intercept val="0"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="8.9119956303785566E-2"/>
+                  <c:y val="3.0948601424649998E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="0"/>
+                      <a:t>Series 1:</a:t>
+                    </a:r>
+                  </a:p>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr/>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>y = 0.2132x</a:t>
+                    </a:r>
+                    <a:br>
+                      <a:rPr lang="en-US" baseline="0"/>
+                    </a:br>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>R² = 0.9984</a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet2!$B$3:$G$3</c:f>
@@ -1085,7 +1149,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4CD0-E548-9EF7-4DBDAF8346F3}"/>
+              <c16:uniqueId val="{00000000-A5BE-8948-B0E0-0E2ED5811E5F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1114,6 +1178,99 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:intercept val="0"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="7.3008361191284649E-2"/>
+                  <c:y val="6.2088225911514298E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="0"/>
+                      <a:t>Series 2:</a:t>
+                    </a:r>
+                  </a:p>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr/>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>y = 0.1951x</a:t>
+                    </a:r>
+                    <a:br>
+                      <a:rPr lang="en-US" baseline="0"/>
+                    </a:br>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>R² = 0.9937</a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet2!$B$3:$G$3</c:f>
@@ -1171,7 +1328,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4CD0-E548-9EF7-4DBDAF8346F3}"/>
+              <c16:uniqueId val="{00000001-A5BE-8948-B0E0-0E2ED5811E5F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1200,6 +1357,99 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:intercept val="0"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="8.0331813515148703E-2"/>
+                  <c:y val="-2.4103608361970875E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="0"/>
+                      <a:t>Series 3:</a:t>
+                    </a:r>
+                  </a:p>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr/>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>y = 0.2374x</a:t>
+                    </a:r>
+                    <a:br>
+                      <a:rPr lang="en-US" baseline="0"/>
+                    </a:br>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>R² = 0.9965</a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet2!$B$3:$G$3</c:f>
@@ -1257,7 +1507,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4CD0-E548-9EF7-4DBDAF8346F3}"/>
+              <c16:uniqueId val="{00000002-A5BE-8948-B0E0-0E2ED5811E5F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1293,6 +1543,68 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Time (minutes)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1355,6 +1667,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="1"/>
+                  <a:t>Weight of melted ice cream (grams)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1405,12 +1772,36 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="b"/>
+      <c:legendPos val="r"/>
+      <c:legendEntry>
+        <c:idx val="3"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:legendEntry>
+        <c:idx val="4"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:legendEntry>
+        <c:idx val="5"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.87896293917936275"/>
+          <c:y val="0.41850144317923504"/>
+          <c:w val="0.11517829896154601"/>
+          <c:h val="0.47837618935734111"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
-        <a:ln>
-          <a:noFill/>
+        <a:ln w="15875">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
         </a:ln>
         <a:effectLst/>
       </c:spPr>
@@ -1419,7 +1810,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1500" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -1471,11 +1862,6 @@
       <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
 </c:chartSpace>
 </file>
 
@@ -3137,6 +3523,14 @@
 </chartsheet>
 </file>
 
+<file path=xl/chartsheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{C0688644-4B6A-0642-AF38-04EE43D0858C}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
@@ -3205,29 +3599,21 @@
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>428074</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>158285</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>57371</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>86890</xdr:rowOff>
-    </xdr:to>
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="8670774" cy="6281964"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09FB373B-C041-F8E4-5D12-D4DAE5600342}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27C4BA7D-24B0-D3AF-9D15-AE83DD2EA614}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -3240,7 +3626,7 @@
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:absoluteAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3663,7 +4049,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Quartz sync: Sep 11, 2025, 12:51 PM
</commit_message>
<xml_diff>
--- a/content/Notes/Biology/Labs/Excel/Lab 1.xlsx
+++ b/content/Notes/Biology/Labs/Excel/Lab 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gassandrid/VAULT/Notes/Biology/Labs/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C820872-849D-C04D-A0F1-673F3CDB534B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45EFB47C-2529-854D-B144-EF90ED728648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="740" windowWidth="34440" windowHeight="21540" activeTab="3" xr2:uid="{16F632E2-7B1C-374A-AA6C-9F513062A785}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
   <si>
     <t>Standard Deviation</t>
   </si>
@@ -119,17 +119,23 @@
   <si>
     <t>Trial #3</t>
   </si>
+  <si>
+    <t>Rate(Grams/Min)</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="168" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -150,6 +156,13 @@
       <name val="Helvetica"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -159,7 +172,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -167,19 +180,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3601,7 +3633,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8670774" cy="6281964"/>
+    <xdr:ext cx="8679682" cy="6293376"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -3947,8 +3979,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A46C606A-3066-9E45-98A0-2DBA9F19BD8B}">
-  <dimension ref="A2:G6"/>
+  <dimension ref="A2:G13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
@@ -4045,6 +4081,54 @@
       </c>
       <c r="G6" s="1">
         <v>13.41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="8"/>
+      <c r="B8" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>0.2132</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10">
+        <v>0.1951</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11">
+        <v>0.2374</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="10">
+        <f>AVERAGE(B9:B11)</f>
+        <v>0.2152333333333333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="11">
+        <f>_xlfn.STDEV.P(B9:B11)</f>
+        <v>1.7328653214321716E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>